<commit_message>
Updated after ADS exam
</commit_message>
<xml_diff>
--- a/Progress-Trackers/Year-1.xlsx
+++ b/Progress-Trackers/Year-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Documents\GitHub\Module-Summaries\Progress-Trackers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FACF85-30E0-44DD-89E6-065F6D0391D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C96DF75-114E-467F-BF86-EEF4F61749B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1A341AAB-498B-4634-A968-4208D8C301AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{1A341AAB-498B-4634-A968-4208D8C301AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphs" sheetId="3" r:id="rId1"/>
@@ -1034,14 +1034,14 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="9" fontId="10" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2070,7 +2070,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -6077,18 +6077,18 @@
       </c>
     </row>
     <row r="10" spans="2:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="R10" s="72" t="s">
+      <c r="R10" s="71" t="s">
         <v>153</v>
       </c>
-      <c r="S10" s="71">
+      <c r="S10" s="70">
         <f>IF(Calculator!F46 &gt; 0, Calculator!F46, "1st Achieved")</f>
         <v>0.6752565974143051</v>
       </c>
-      <c r="T10" s="71" cm="1">
+      <c r="T10" s="70" cm="1">
         <f t="array" ref="T10">_xlfn.IFS(S10="1st Achieved", "-", Calculator!G46 &gt; 0, Calculator!G46, TRUE, "2:1 Achieved")</f>
         <v>0.50284280431085693</v>
       </c>
-      <c r="U10" s="71" cm="1">
+      <c r="U10" s="70" cm="1">
         <f t="array" ref="U10">_xlfn.IFS(T10="-", "-", T10="2:1 Achieved", "-", Calculator!H46 &gt; 0, Calculator!H46, TRUE, "Passed")</f>
         <v>0.3304290112074087</v>
       </c>
@@ -6843,26 +6843,26 @@
       <c r="AG23" s="14"/>
     </row>
     <row r="25" spans="2:33" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="70" t="str">
+      <c r="B25" s="72" t="str">
         <f ca="1">SUM(Calculator!L31:L36) &amp; " summatives completed this academic year. (Average: " &amp; ROUND(AVERAGEIF(Calculator!P31:P36, "&gt;0"),2)*100 &amp; "%)"</f>
-        <v>13 summatives completed this academic year. (Average: 77%)</v>
-      </c>
-      <c r="C25" s="70"/>
-      <c r="D25" s="70"/>
-      <c r="E25" s="70"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="70"/>
-      <c r="J25" s="70" t="str">
+        <v>14 summatives completed this academic year. (Average: 77%)</v>
+      </c>
+      <c r="C25" s="72"/>
+      <c r="D25" s="72"/>
+      <c r="E25" s="72"/>
+      <c r="F25" s="72"/>
+      <c r="G25" s="72"/>
+      <c r="H25" s="72"/>
+      <c r="J25" s="72" t="str">
         <f ca="1">SUM(Calculator!D31:D36) &amp; " formatives completed this academic year. (Average: " &amp; ROUND(AVERAGEIF(Calculator!H31:H36, "&gt;0"),2)*100 &amp; "%)"</f>
         <v>26 formatives completed this academic year. (Average: 80%)</v>
       </c>
-      <c r="K25" s="70"/>
-      <c r="L25" s="70"/>
-      <c r="M25" s="70"/>
-      <c r="N25" s="70"/>
-      <c r="O25" s="70"/>
-      <c r="P25" s="70"/>
+      <c r="K25" s="72"/>
+      <c r="L25" s="72"/>
+      <c r="M25" s="72"/>
+      <c r="N25" s="72"/>
+      <c r="O25" s="72"/>
+      <c r="P25" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10635,7 +10635,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A2" ca="1">_xlfn.IFS(H2, "Done", B2 &gt; NOW(), "Not Released", C2 &lt; NOW(), "Overdue", TRUE, ROUND(C2 - NOW(), 1) &amp; " Days")</f>
-        <v>18.2 Days</v>
+        <v>12.1 Days</v>
       </c>
       <c r="B2" s="27">
         <v>46093</v>
@@ -10670,7 +10670,7 @@
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A3" ca="1">_xlfn.IFS(H3, "Done", B3 &gt; NOW(), "Not Released", C3 &lt; NOW(), "Overdue", TRUE, ROUND(C3 - NOW(), 1) &amp; " Days")</f>
-        <v>13.2 Days</v>
+        <v>7.1 Days</v>
       </c>
       <c r="B3" s="27">
         <v>46093</v>
@@ -10718,7 +10718,7 @@
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A4" ca="1">_xlfn.IFS(H4, "Done", B4 &gt; NOW(), "Not Released", C4 &lt; NOW(), "Overdue", TRUE, ROUND(C4 - NOW(), 1) &amp; " Days")</f>
-        <v>7.2 Days</v>
+        <v>1.1 Days</v>
       </c>
       <c r="B4" s="27">
         <v>46093</v>
@@ -10766,7 +10766,7 @@
     <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A5" ca="1">_xlfn.IFS(H5, "Done", B5 &gt; NOW(), "Not Released", C5 &lt; NOW(), "Overdue", TRUE, ROUND(C5 - NOW(), 1) &amp; " Days")</f>
-        <v>5.2 Days</v>
+        <v>Done</v>
       </c>
       <c r="B5" s="27">
         <v>46093</v>
@@ -10787,7 +10787,7 @@
         <v>75</v>
       </c>
       <c r="H5" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="44"/>
       <c r="J5" s="41">
@@ -14283,7 +14283,7 @@
       </c>
       <c r="L31">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B31, 'Summatives Tracker'!$A$2:$A$1004, "Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B31, 'Summatives Tracker'!$A$2:$A$1004, "Not Released")</f>
@@ -14291,11 +14291,11 @@
       </c>
       <c r="N31">
         <f ca="1">K31-L31-M31</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31">
         <f ca="1">K31-L31</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P31" s="2">
         <f>IFERROR(AVERAGEIF('Summatives Tracker'!$E$6:$E$1004, $B31, 'Summatives Tracker'!$I$6:$I$1004), 0)</f>
@@ -14673,7 +14673,7 @@
         <v>0</v>
       </c>
       <c r="I41" s="47">
-        <f t="shared" ref="I41:I46" si="51">IFERROR(IF((0.4-$C41)/$E41&gt;0,(0.4-$C41)/$E41,0), IF($C41&gt;=0.4, 0, 1))</f>
+        <f t="shared" ref="I41:I45" si="51">IFERROR(IF((0.4-$C41)/$E41&gt;0,(0.4-$C41)/$E41,0), IF($C41&gt;=0.4, 0, 1))</f>
         <v>0</v>
       </c>
     </row>
@@ -14694,7 +14694,7 @@
         <v>0.66</v>
       </c>
       <c r="F42" s="47">
-        <f t="shared" ref="F42:F46" si="52">IFERROR(IF((0.7-$C42)/$E42&gt;0,(0.7-$C42)/$E42,0), IF($C42&gt;=0.7, 0, 1))</f>
+        <f t="shared" ref="F42:F45" si="52">IFERROR(IF((0.7-$C42)/$E42&gt;0,(0.7-$C42)/$E42,0), IF($C42&gt;=0.7, 0, 1))</f>
         <v>0.63174242424242411</v>
       </c>
       <c r="G42" s="47">

</xml_diff>

<commit_message>
Updated Year 1 Grades
</commit_message>
<xml_diff>
--- a/Progress-Trackers/Year-1.xlsx
+++ b/Progress-Trackers/Year-1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Documents\GitHub\Module-Summaries\Progress-Trackers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C96DF75-114E-467F-BF86-EEF4F61749B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7180D541-2539-43A0-9373-ACB0FD01D256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{1A341AAB-498B-4634-A968-4208D8C301AA}"/>
   </bookViews>
@@ -1378,7 +1378,7 @@
                   <c:v>0.72499999999999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.83499999999999996</c:v>
+                  <c:v>0.79333333333333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2076,13 +2076,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -2344,10 +2344,10 @@
                   <c:v>0.2465</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.35150000000000003</c:v>
+                  <c:v>0.70650000000000002</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.30835117349970292</c:v>
+                  <c:v>0.36751784016636962</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2435,10 +2435,10 @@
                   <c:v>0.34</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.5</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.41999999999999993</c:v>
+                  <c:v>0.5033333333333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5954,7 +5954,7 @@
     <row r="2" spans="2:33" x14ac:dyDescent="0.35">
       <c r="B2" s="15" t="str">
         <f>"Achieved vs. Possible Module Scores (" &amp; ROUND(AVERAGEIF(Calculator!D40:D45, "&gt;0", Calculator!C40:C45)*100, 0) &amp; "%  vs.  " &amp; ROUND(AVERAGEIF(Calculator!D40:D45, "&gt;0")*100, 0) &amp; "%, " &amp; ROUND((AVERAGEIF(Calculator!D40:D45, "&gt;0", Calculator!C40:C45)/AVERAGEIF(Calculator!D40:D45, "&gt;0"))*100,0) &amp; "% Average)"</f>
-        <v>Achieved vs. Possible Module Scores (37%  vs.  50%, 73% Average)</v>
+        <v>Achieved vs. Possible Module Scores (44%  vs.  60%, 73% Average)</v>
       </c>
       <c r="R2" s="20" t="s">
         <v>149</v>
@@ -6063,17 +6063,17 @@
       <c r="R9" s="67" t="s">
         <v>147</v>
       </c>
-      <c r="S9" s="66">
+      <c r="S9" s="66" t="str">
         <f>IF(Calculator!F45 &gt; 0, Calculator!F45, "1st Achieved")</f>
-        <v>0.69699999999999984</v>
-      </c>
-      <c r="T9" s="66" cm="1">
+        <v>1st Achieved</v>
+      </c>
+      <c r="T9" s="66" t="str" cm="1">
         <f t="array" ref="T9">_xlfn.IFS(S9="1st Achieved", "-", Calculator!G45 &gt; 0, Calculator!G45, TRUE, "2:1 Achieved")</f>
-        <v>0.49699999999999989</v>
-      </c>
-      <c r="U9" s="66" cm="1">
+        <v>-</v>
+      </c>
+      <c r="U9" s="66" t="str" cm="1">
         <f t="array" ref="U9">_xlfn.IFS(T9="-", "-", T9="2:1 Achieved", "-", Calculator!H45 &gt; 0, Calculator!H45, TRUE, "Passed")</f>
-        <v>0.29699999999999993</v>
+        <v>-</v>
       </c>
     </row>
     <row r="10" spans="2:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -6082,15 +6082,15 @@
       </c>
       <c r="S10" s="70">
         <f>IF(Calculator!F46 &gt; 0, Calculator!F46, "1st Achieved")</f>
-        <v>0.6752565974143051</v>
+        <v>0.66942716745026232</v>
       </c>
       <c r="T10" s="70" cm="1">
         <f t="array" ref="T10">_xlfn.IFS(S10="1st Achieved", "-", Calculator!G46 &gt; 0, Calculator!G46, TRUE, "2:1 Achieved")</f>
-        <v>0.50284280431085693</v>
+        <v>0.46808488557106775</v>
       </c>
       <c r="U10" s="70" cm="1">
         <f t="array" ref="U10">_xlfn.IFS(T10="-", "-", T10="2:1 Achieved", "-", Calculator!H46 &gt; 0, Calculator!H46, TRUE, "Passed")</f>
-        <v>0.3304290112074087</v>
+        <v>0.26674260369187319</v>
       </c>
     </row>
     <row r="11" spans="2:33" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
@@ -6845,7 +6845,7 @@
     <row r="25" spans="2:33" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="72" t="str">
         <f ca="1">SUM(Calculator!L31:L36) &amp; " summatives completed this academic year. (Average: " &amp; ROUND(AVERAGEIF(Calculator!P31:P36, "&gt;0"),2)*100 &amp; "%)"</f>
-        <v>14 summatives completed this academic year. (Average: 77%)</v>
+        <v>17 summatives completed this academic year. (Average: 77%)</v>
       </c>
       <c r="C25" s="72"/>
       <c r="D25" s="72"/>
@@ -10635,7 +10635,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A2" ca="1">_xlfn.IFS(H2, "Done", B2 &gt; NOW(), "Not Released", C2 &lt; NOW(), "Overdue", TRUE, ROUND(C2 - NOW(), 1) &amp; " Days")</f>
-        <v>12.1 Days</v>
+        <v>Done</v>
       </c>
       <c r="B2" s="27">
         <v>46093</v>
@@ -10656,7 +10656,7 @@
         <v>75</v>
       </c>
       <c r="H2" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="44"/>
       <c r="J2" s="41">
@@ -10670,7 +10670,7 @@
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A3" ca="1">_xlfn.IFS(H3, "Done", B3 &gt; NOW(), "Not Released", C3 &lt; NOW(), "Overdue", TRUE, ROUND(C3 - NOW(), 1) &amp; " Days")</f>
-        <v>7.1 Days</v>
+        <v>Done</v>
       </c>
       <c r="B3" s="27">
         <v>46093</v>
@@ -10691,7 +10691,7 @@
         <v>75</v>
       </c>
       <c r="H3" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" s="44"/>
       <c r="J3" s="41">
@@ -10718,7 +10718,7 @@
     <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A4" ca="1">_xlfn.IFS(H4, "Done", B4 &gt; NOW(), "Not Released", C4 &lt; NOW(), "Overdue", TRUE, ROUND(C4 - NOW(), 1) &amp; " Days")</f>
-        <v>1.1 Days</v>
+        <v>Done</v>
       </c>
       <c r="B4" s="27">
         <v>46093</v>
@@ -10739,7 +10739,7 @@
         <v>75</v>
       </c>
       <c r="H4" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="44"/>
       <c r="J4" s="41">
@@ -10837,13 +10837,15 @@
       <c r="H6" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="I6" s="44"/>
+      <c r="I6" s="44">
+        <v>0.71</v>
+      </c>
       <c r="J6" s="41">
         <v>0.5</v>
       </c>
       <c r="K6" s="45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.35499999999999998</v>
       </c>
       <c r="N6" s="29"/>
       <c r="O6" s="30"/>
@@ -14395,7 +14397,7 @@
       </c>
       <c r="L33">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B33, 'Summatives Tracker'!$A$2:$A$1004, "Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M33">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B33, 'Summatives Tracker'!$A$2:$A$1004, "Not Released")</f>
@@ -14403,11 +14405,11 @@
       </c>
       <c r="N33">
         <f t="shared" ca="1" si="46"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O33">
         <f t="shared" ca="1" si="47"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P33" s="2">
         <f>IFERROR(AVERAGEIF('Summatives Tracker'!$E$6:$E$1004, $B33, 'Summatives Tracker'!$I$6:$I$1004), 0)</f>
@@ -14451,7 +14453,7 @@
       </c>
       <c r="L34">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B34, 'Summatives Tracker'!$A$2:$A$1004, "Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M34">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B34, 'Summatives Tracker'!$A$2:$A$1004, "Not Released")</f>
@@ -14459,11 +14461,11 @@
       </c>
       <c r="N34">
         <f t="shared" ca="1" si="46"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O34">
         <f t="shared" ca="1" si="47"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P34" s="2">
         <f>IFERROR(AVERAGEIF('Summatives Tracker'!$E$6:$E$1004, $B34, 'Summatives Tracker'!$I$6:$I$1004), 0)</f>
@@ -14507,7 +14509,7 @@
       </c>
       <c r="L35">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B35, 'Summatives Tracker'!$A$2:$A$1004, "Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M35">
         <f ca="1">COUNTIFS('Summatives Tracker'!$E$2:$E$1004, $B35, 'Summatives Tracker'!$A$2:$A$1004, "Not Released")</f>
@@ -14515,11 +14517,11 @@
       </c>
       <c r="N35">
         <f t="shared" ca="1" si="46"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O35">
         <f t="shared" ca="1" si="47"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P35" s="2">
         <f>IFERROR(AVERAGEIF('Summatives Tracker'!$E$6:$E$1004, $B35, 'Summatives Tracker'!$I$6:$I$1004), 0)</f>
@@ -14579,7 +14581,7 @@
       </c>
       <c r="P36" s="2">
         <f>IFERROR(AVERAGEIF('Summatives Tracker'!$E$6:$E$1004, $B36, 'Summatives Tracker'!$I$6:$I$1004), 0)</f>
-        <v>0.83499999999999996</v>
+        <v>0.79333333333333333</v>
       </c>
     </row>
     <row r="38" spans="2:16" x14ac:dyDescent="0.35">
@@ -14782,31 +14784,31 @@
       </c>
       <c r="C45" s="46">
         <f>IFERROR(SUMIF('Summatives Tracker'!$E$2:$E$1004, $B45, 'Summatives Tracker'!$K$2:$K$1004), 0)</f>
-        <v>0.35150000000000003</v>
+        <v>0.70650000000000002</v>
       </c>
       <c r="D45" s="46">
         <f>SUMIFS('Summatives Tracker'!$J$2:$J$1003, 'Summatives Tracker'!$I$2:$I$1003, "&gt;0", 'Summatives Tracker'!$E$2:$E$1003, B45)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E45" s="47">
         <f t="shared" si="48"/>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F45" s="47">
         <f t="shared" si="52"/>
-        <v>0.69699999999999984</v>
+        <v>0</v>
       </c>
       <c r="G45" s="47">
         <f t="shared" si="49"/>
-        <v>0.49699999999999989</v>
+        <v>0</v>
       </c>
       <c r="H45" s="47">
         <f t="shared" si="50"/>
-        <v>0.29699999999999993</v>
+        <v>0</v>
       </c>
       <c r="I45" s="47">
         <f t="shared" si="51"/>
-        <v>9.6999999999999975E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="2:16" x14ac:dyDescent="0.35">
@@ -14815,31 +14817,31 @@
       </c>
       <c r="C46" s="47">
         <f>SUM(C40:C45)/6</f>
-        <v>0.30835117349970292</v>
+        <v>0.36751784016636962</v>
       </c>
       <c r="D46" s="47">
         <f>SUM(D40:D45)/6</f>
-        <v>0.41999999999999993</v>
+        <v>0.5033333333333333</v>
       </c>
       <c r="E46" s="47">
         <f>SUM(E40:E45)/6</f>
-        <v>0.58000000000000007</v>
+        <v>0.49666666666666676</v>
       </c>
       <c r="F46" s="47">
         <f>IFERROR(IF((0.7-$C46)/$E46&gt;0,(0.7-$C46)/$E46,0), IF($C46&gt;=0.7, 0, 1))</f>
-        <v>0.6752565974143051</v>
+        <v>0.66942716745026232</v>
       </c>
       <c r="G46" s="47">
         <f t="shared" si="49"/>
-        <v>0.50284280431085693</v>
+        <v>0.46808488557106775</v>
       </c>
       <c r="H46" s="47">
         <f t="shared" si="50"/>
-        <v>0.3304290112074087</v>
+        <v>0.26674260369187319</v>
       </c>
       <c r="I46" s="47">
         <f>IFERROR(IF((0.4-$C46)/$E46&gt;0,(0.4-$C46)/$E46,0), IF($C46&gt;=0.4, 0, 1))</f>
-        <v>0.15801521810396049</v>
+        <v>6.5400321812678644E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added some exam scores
</commit_message>
<xml_diff>
--- a/Progress-Trackers/Year-1.xlsx
+++ b/Progress-Trackers/Year-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Documents\GitHub\Module-Summaries\Progress-Trackers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7180D541-2539-43A0-9373-ACB0FD01D256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF53243-DC9F-45EF-BAD9-8EEA882DC659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{1A341AAB-498B-4634-A968-4208D8C301AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1A341AAB-498B-4634-A968-4208D8C301AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphs" sheetId="3" r:id="rId1"/>
@@ -1372,7 +1372,7 @@
                   <c:v>0.83250000000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.55000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.72499999999999998</c:v>
@@ -1834,7 +1834,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2335,19 +2335,19 @@
                   <c:v>0.71405704099821754</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.28305000000000002</c:v>
+                  <c:v>0.60315000000000007</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.55000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.2465</c:v>
+                  <c:v>0.60289999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0.70650000000000002</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.36751784016636962</c:v>
+                  <c:v>0.57193450683303626</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2426,19 +2426,19 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.33999999999999997</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.99999999999999989</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.34</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.5033333333333333</c:v>
+                  <c:v>0.89</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5954,7 +5954,7 @@
     <row r="2" spans="2:33" x14ac:dyDescent="0.35">
       <c r="B2" s="15" t="str">
         <f>"Achieved vs. Possible Module Scores (" &amp; ROUND(AVERAGEIF(Calculator!D40:D45, "&gt;0", Calculator!C40:C45)*100, 0) &amp; "%  vs.  " &amp; ROUND(AVERAGEIF(Calculator!D40:D45, "&gt;0")*100, 0) &amp; "%, " &amp; ROUND((AVERAGEIF(Calculator!D40:D45, "&gt;0", Calculator!C40:C45)/AVERAGEIF(Calculator!D40:D45, "&gt;0"))*100,0) &amp; "% Average)"</f>
-        <v>Achieved vs. Possible Module Scores (44%  vs.  60%, 73% Average)</v>
+        <v>Achieved vs. Possible Module Scores (57%  vs.  89%, 64% Average)</v>
       </c>
       <c r="R2" s="20" t="s">
         <v>149</v>
@@ -6014,15 +6014,15 @@
       </c>
       <c r="S6" s="66">
         <f>IF(Calculator!F42 &gt; 0, Calculator!F42, "1st Achieved")</f>
-        <v>0.63174242424242411</v>
-      </c>
-      <c r="T6" s="66" cm="1">
+        <v>1</v>
+      </c>
+      <c r="T6" s="66" t="str" cm="1">
         <f t="array" ref="T6">_xlfn.IFS(S6="1st Achieved", "-", Calculator!G42 &gt; 0, Calculator!G42, TRUE, "2:1 Achieved")</f>
-        <v>0.48022727272727261</v>
-      </c>
-      <c r="U6" s="66" cm="1">
+        <v>2:1 Achieved</v>
+      </c>
+      <c r="U6" s="66" t="str" cm="1">
         <f t="array" ref="U6">_xlfn.IFS(T6="-", "-", T6="2:1 Achieved", "-", Calculator!H42 &gt; 0, Calculator!H42, TRUE, "Passed")</f>
-        <v>0.32871212121212118</v>
+        <v>-</v>
       </c>
     </row>
     <row r="7" spans="2:33" x14ac:dyDescent="0.35">
@@ -6031,15 +6031,15 @@
       </c>
       <c r="S7" s="66">
         <f>IF(Calculator!F43 &gt; 0, Calculator!F43, "1st Achieved")</f>
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="T7" s="66" cm="1">
         <f t="array" ref="T7">_xlfn.IFS(S7="1st Achieved", "-", Calculator!G43 &gt; 0, Calculator!G43, TRUE, "2:1 Achieved")</f>
-        <v>0.6</v>
-      </c>
-      <c r="U7" s="66" cm="1">
+        <v>1</v>
+      </c>
+      <c r="U7" s="66" t="str" cm="1">
         <f t="array" ref="U7">_xlfn.IFS(T7="-", "-", T7="2:1 Achieved", "-", Calculator!H43 &gt; 0, Calculator!H43, TRUE, "Passed")</f>
-        <v>0.5</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="8" spans="2:33" x14ac:dyDescent="0.35">
@@ -6048,15 +6048,15 @@
       </c>
       <c r="S8" s="66">
         <f>IF(Calculator!F44 &gt; 0, Calculator!F44, "1st Achieved")</f>
-        <v>0.68712121212121213</v>
-      </c>
-      <c r="T8" s="66" cm="1">
+        <v>1</v>
+      </c>
+      <c r="T8" s="66" t="str" cm="1">
         <f t="array" ref="T8">_xlfn.IFS(S8="1st Achieved", "-", Calculator!G44 &gt; 0, Calculator!G44, TRUE, "2:1 Achieved")</f>
-        <v>0.53560606060606064</v>
-      </c>
-      <c r="U8" s="66" cm="1">
+        <v>2:1 Achieved</v>
+      </c>
+      <c r="U8" s="66" t="str" cm="1">
         <f t="array" ref="U8">_xlfn.IFS(T8="-", "-", T8="2:1 Achieved", "-", Calculator!H44 &gt; 0, Calculator!H44, TRUE, "Passed")</f>
-        <v>0.38409090909090915</v>
+        <v>-</v>
       </c>
     </row>
     <row r="9" spans="2:33" x14ac:dyDescent="0.35">
@@ -6082,15 +6082,15 @@
       </c>
       <c r="S10" s="70">
         <f>IF(Calculator!F46 &gt; 0, Calculator!F46, "1st Achieved")</f>
-        <v>0.66942716745026232</v>
+        <v>1.1642317560633064</v>
       </c>
       <c r="T10" s="70" cm="1">
         <f t="array" ref="T10">_xlfn.IFS(S10="1st Achieved", "-", Calculator!G46 &gt; 0, Calculator!G46, TRUE, "2:1 Achieved")</f>
-        <v>0.46808488557106775</v>
-      </c>
-      <c r="U10" s="70" cm="1">
+        <v>0.25514084697239742</v>
+      </c>
+      <c r="U10" s="70" t="str" cm="1">
         <f t="array" ref="U10">_xlfn.IFS(T10="-", "-", T10="2:1 Achieved", "-", Calculator!H46 &gt; 0, Calculator!H46, TRUE, "Passed")</f>
-        <v>0.26674260369187319</v>
+        <v>Passed</v>
       </c>
     </row>
     <row r="11" spans="2:33" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
@@ -6845,7 +6845,7 @@
     <row r="25" spans="2:33" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="72" t="str">
         <f ca="1">SUM(Calculator!L31:L36) &amp; " summatives completed this academic year. (Average: " &amp; ROUND(AVERAGEIF(Calculator!P31:P36, "&gt;0"),2)*100 &amp; "%)"</f>
-        <v>17 summatives completed this academic year. (Average: 77%)</v>
+        <v>17 summatives completed this academic year. (Average: 73%)</v>
       </c>
       <c r="C25" s="72"/>
       <c r="D25" s="72"/>
@@ -6855,7 +6855,7 @@
       <c r="H25" s="72"/>
       <c r="J25" s="72" t="str">
         <f ca="1">SUM(Calculator!D31:D36) &amp; " formatives completed this academic year. (Average: " &amp; ROUND(AVERAGEIF(Calculator!H31:H36, "&gt;0"),2)*100 &amp; "%)"</f>
-        <v>26 formatives completed this academic year. (Average: 80%)</v>
+        <v>27 formatives completed this academic year. (Average: 80%)</v>
       </c>
       <c r="K25" s="72"/>
       <c r="L25" s="72"/>
@@ -9199,7 +9199,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="42" t="str" cm="1">
         <f t="array" aca="1" ref="A2" ca="1">_xlfn.IFS(H2, "Done", B2 &gt; NOW(), "Not Released", C2 &lt; NOW(), "Overdue", TRUE, ROUND(C2 - NOW(), 1) &amp; " Days")</f>
-        <v>Overdue</v>
+        <v>Done</v>
       </c>
       <c r="B2" s="27">
         <v>45996</v>
@@ -9220,7 +9220,7 @@
         <v>71</v>
       </c>
       <c r="H2" s="28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="41"/>
       <c r="J2" s="41" t="str" cm="1">
@@ -10658,13 +10658,15 @@
       <c r="H2" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="I2" s="44"/>
+      <c r="I2" s="44">
+        <v>0.55000000000000004</v>
+      </c>
       <c r="J2" s="41">
         <v>0.7</v>
       </c>
       <c r="K2" s="45">
         <f t="shared" ref="K2:K18" si="0">J2*I2</f>
-        <v>0</v>
+        <v>0.38500000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.35">
@@ -10693,13 +10695,15 @@
       <c r="H3" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="I3" s="44"/>
+      <c r="I3" s="44">
+        <v>0.54</v>
+      </c>
       <c r="J3" s="41">
         <v>0.66</v>
       </c>
       <c r="K3" s="45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.35640000000000005</v>
       </c>
       <c r="N3" s="29"/>
       <c r="O3" s="30"/>
@@ -10741,13 +10745,15 @@
       <c r="H4" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="I4" s="44"/>
+      <c r="I4" s="44">
+        <v>0.48499999999999999</v>
+      </c>
       <c r="J4" s="41">
         <v>0.66</v>
       </c>
       <c r="K4" s="45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.3201</v>
       </c>
       <c r="N4" s="29"/>
       <c r="O4" s="30"/>
@@ -10939,13 +10945,15 @@
       <c r="H8" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="I8" s="44"/>
+      <c r="I8" s="44">
+        <v>0.55000000000000004</v>
+      </c>
       <c r="J8" s="41">
         <v>0.2</v>
       </c>
       <c r="K8" s="45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.11000000000000001</v>
       </c>
       <c r="N8" s="29"/>
       <c r="O8" s="30"/>
@@ -11039,13 +11047,15 @@
       <c r="H10" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="I10" s="44"/>
+      <c r="I10" s="44">
+        <v>0.55000000000000004</v>
+      </c>
       <c r="J10" s="41">
         <v>0.1</v>
       </c>
       <c r="K10" s="45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5.5000000000000007E-2</v>
       </c>
       <c r="N10" s="29"/>
       <c r="O10" s="30"/>
@@ -14426,7 +14436,7 @@
       </c>
       <c r="D34">
         <f ca="1">COUNTIFS('Formatives Tracker'!$E$2:$E$1008, $B34, 'Formatives Tracker'!$A$2:$A$1008, "Done")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E34">
         <f ca="1">COUNTIFS('Formatives Tracker'!$E$2:$E$1008, $B34, 'Formatives Tracker'!$A$2:$A$1008, "Not Released")</f>
@@ -14434,11 +14444,11 @@
       </c>
       <c r="F34">
         <f t="shared" ca="1" si="44"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34">
         <f t="shared" ca="1" si="45"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H34" s="2">
         <f>IFERROR(AVERAGEIF('Formatives Tracker'!$E$2:$E$1008, $B34, 'Formatives Tracker'!$J$2:$J$1008), 0)</f>
@@ -14469,7 +14479,7 @@
       </c>
       <c r="P34" s="2">
         <f>IFERROR(AVERAGEIF('Summatives Tracker'!$E$6:$E$1004, $B34, 'Summatives Tracker'!$I$6:$I$1004), 0)</f>
-        <v>0</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="35" spans="2:16" x14ac:dyDescent="0.35">
@@ -14630,19 +14640,19 @@
         <v>0.66</v>
       </c>
       <c r="F40" s="47">
-        <f>IFERROR(IF((0.7-$C40)/$E40&gt;0,(0.7-$C40)/$E40,0), IF($C40&gt;=0.7, 0, 1))</f>
+        <f>IFERROR(IF((0.7-$C40)/$E40&gt;=0,(0.7-$C40)/$E40,0), IF($C40&gt;=0.7, 0, 1))</f>
         <v>0.67424242424242409</v>
       </c>
       <c r="G40" s="47">
-        <f>IFERROR(IF((0.6-$C40)/$E40&gt;0,(0.6-$C40)/$E40,0), IF($C40&gt;=0.6, 0, 1))</f>
+        <f>IFERROR(IF((0.6-$C40)/$E40&gt;=0,(0.6-$C40)/$E40,0), IF($C40&gt;=0.6, 0, 1))</f>
         <v>0.52272727272727271</v>
       </c>
       <c r="H40" s="47">
-        <f>IFERROR(IF((0.5-$C40)/$E40&gt;0,(0.5-$C40)/$E40,0), IF($C40&gt;=0.5, 0, 1))</f>
+        <f>IFERROR(IF((0.5-$C40)/$E40&gt;=0,(0.5-$C40)/$E40,0), IF($C40&gt;=0.5, 0, 1))</f>
         <v>0.37121212121212122</v>
       </c>
       <c r="I40" s="47">
-        <f>IFERROR(IF((0.4-$C40)/$E40&gt;0,(0.4-$C40)/$E40,0), IF($C40&gt;=0.4, 0, 1))</f>
+        <f>IFERROR(IF((0.4-$C40)/$E40&gt;=0,(0.4-$C40)/$E40,0), IF($C40&gt;=0.4, 0, 1))</f>
         <v>0.21969696969696972</v>
       </c>
     </row>
@@ -14663,19 +14673,19 @@
         <v>0</v>
       </c>
       <c r="F41" s="47">
-        <f>IFERROR(IF((0.7-$C41)/$E41&gt;0,(0.7-$C41)/$E41,0), IF($C41&gt;=0.7, 0, 1))</f>
+        <f t="shared" ref="F41:F46" si="49">IFERROR(IF((0.7-$C41)/$E41&gt;=0,(0.7-$C41)/$E41,0), IF($C41&gt;=0.7, 0, 1))</f>
         <v>0</v>
       </c>
       <c r="G41" s="47">
-        <f t="shared" ref="G41:G46" si="49">IFERROR(IF((0.6-$C41)/$E41&gt;0,(0.6-$C41)/$E41,0), IF($C41&gt;=0.6, 0, 1))</f>
+        <f t="shared" ref="G41:G46" si="50">IFERROR(IF((0.6-$C41)/$E41&gt;=0,(0.6-$C41)/$E41,0), IF($C41&gt;=0.6, 0, 1))</f>
         <v>0</v>
       </c>
       <c r="H41" s="47">
-        <f t="shared" ref="H41:H46" si="50">IFERROR(IF((0.5-$C41)/$E41&gt;0,(0.5-$C41)/$E41,0), IF($C41&gt;=0.5, 0, 1))</f>
+        <f t="shared" ref="H41:H46" si="51">IFERROR(IF((0.5-$C41)/$E41&gt;=0,(0.5-$C41)/$E41,0), IF($C41&gt;=0.5, 0, 1))</f>
         <v>0</v>
       </c>
       <c r="I41" s="47">
-        <f t="shared" ref="I41:I45" si="51">IFERROR(IF((0.4-$C41)/$E41&gt;0,(0.4-$C41)/$E41,0), IF($C41&gt;=0.4, 0, 1))</f>
+        <f t="shared" ref="I41:I46" si="52">IFERROR(IF((0.4-$C41)/$E41&gt;=0,(0.4-$C41)/$E41,0), IF($C41&gt;=0.4, 0, 1))</f>
         <v>0</v>
       </c>
     </row>
@@ -14685,31 +14695,31 @@
       </c>
       <c r="C42" s="46">
         <f>IFERROR(SUMIF('Summatives Tracker'!$E$2:$E$1004, $B42, 'Summatives Tracker'!$K$2:$K$1004), 0)</f>
-        <v>0.28305000000000002</v>
+        <v>0.60315000000000007</v>
       </c>
       <c r="D42" s="46">
         <f>SUMIFS('Summatives Tracker'!$J$2:$J$1003, 'Summatives Tracker'!$I$2:$I$1003, "&gt;0", 'Summatives Tracker'!$E$2:$E$1003, B42)</f>
-        <v>0.33999999999999997</v>
+        <v>1</v>
       </c>
       <c r="E42" s="47">
         <f t="shared" si="48"/>
-        <v>0.66</v>
+        <v>0</v>
       </c>
       <c r="F42" s="47">
-        <f t="shared" ref="F42:F45" si="52">IFERROR(IF((0.7-$C42)/$E42&gt;0,(0.7-$C42)/$E42,0), IF($C42&gt;=0.7, 0, 1))</f>
-        <v>0.63174242424242411</v>
+        <f t="shared" si="49"/>
+        <v>1</v>
       </c>
       <c r="G42" s="47">
-        <f t="shared" si="49"/>
-        <v>0.48022727272727261</v>
+        <f t="shared" si="50"/>
+        <v>0</v>
       </c>
       <c r="H42" s="47">
-        <f t="shared" si="50"/>
-        <v>0.32871212121212118</v>
+        <f t="shared" si="51"/>
+        <v>0</v>
       </c>
       <c r="I42" s="47">
-        <f t="shared" si="51"/>
-        <v>0.17719696969696969</v>
+        <f t="shared" si="52"/>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="2:16" x14ac:dyDescent="0.35">
@@ -14718,31 +14728,31 @@
       </c>
       <c r="C43" s="46">
         <f>IFERROR(SUMIF('Summatives Tracker'!$E$2:$E$1004, $B43, 'Summatives Tracker'!$K$2:$K$1004), 0)</f>
-        <v>0</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="D43" s="46">
         <f>SUMIFS('Summatives Tracker'!$J$2:$J$1003, 'Summatives Tracker'!$I$2:$I$1003, "&gt;0", 'Summatives Tracker'!$E$2:$E$1003, B43)</f>
-        <v>0</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="E43" s="47">
         <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="F43" s="47">
+        <f t="shared" si="49"/>
         <v>1</v>
       </c>
-      <c r="F43" s="47">
+      <c r="G43" s="47">
+        <f t="shared" si="50"/>
+        <v>1</v>
+      </c>
+      <c r="H43" s="47">
+        <f t="shared" si="51"/>
+        <v>0</v>
+      </c>
+      <c r="I43" s="47">
         <f t="shared" si="52"/>
-        <v>0.7</v>
-      </c>
-      <c r="G43" s="47">
-        <f t="shared" si="49"/>
-        <v>0.6</v>
-      </c>
-      <c r="H43" s="47">
-        <f t="shared" si="50"/>
-        <v>0.5</v>
-      </c>
-      <c r="I43" s="47">
-        <f t="shared" si="51"/>
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="2:16" x14ac:dyDescent="0.35">
@@ -14751,31 +14761,31 @@
       </c>
       <c r="C44" s="46">
         <f>IFERROR(SUMIF('Summatives Tracker'!$E$2:$E$1004, $B44, 'Summatives Tracker'!$K$2:$K$1004), 0)</f>
-        <v>0.2465</v>
+        <v>0.60289999999999999</v>
       </c>
       <c r="D44" s="46">
         <f>SUMIFS('Summatives Tracker'!$J$2:$J$1003, 'Summatives Tracker'!$I$2:$I$1003, "&gt;0", 'Summatives Tracker'!$E$2:$E$1003, B44)</f>
-        <v>0.34</v>
+        <v>1</v>
       </c>
       <c r="E44" s="47">
         <f t="shared" si="48"/>
-        <v>0.65999999999999992</v>
+        <v>0</v>
       </c>
       <c r="F44" s="47">
+        <f t="shared" si="49"/>
+        <v>1</v>
+      </c>
+      <c r="G44" s="47">
+        <f t="shared" si="50"/>
+        <v>0</v>
+      </c>
+      <c r="H44" s="47">
+        <f t="shared" si="51"/>
+        <v>0</v>
+      </c>
+      <c r="I44" s="47">
         <f t="shared" si="52"/>
-        <v>0.68712121212121213</v>
-      </c>
-      <c r="G44" s="47">
-        <f t="shared" si="49"/>
-        <v>0.53560606060606064</v>
-      </c>
-      <c r="H44" s="47">
-        <f t="shared" si="50"/>
-        <v>0.38409090909090915</v>
-      </c>
-      <c r="I44" s="47">
-        <f t="shared" si="51"/>
-        <v>0.23257575757575763</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="2:16" x14ac:dyDescent="0.35">
@@ -14795,19 +14805,19 @@
         <v>0</v>
       </c>
       <c r="F45" s="47">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="G45" s="47">
+        <f t="shared" si="50"/>
+        <v>0</v>
+      </c>
+      <c r="H45" s="47">
+        <f t="shared" si="51"/>
+        <v>0</v>
+      </c>
+      <c r="I45" s="47">
         <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="G45" s="47">
-        <f t="shared" si="49"/>
-        <v>0</v>
-      </c>
-      <c r="H45" s="47">
-        <f t="shared" si="50"/>
-        <v>0</v>
-      </c>
-      <c r="I45" s="47">
-        <f t="shared" si="51"/>
         <v>0</v>
       </c>
     </row>
@@ -14817,31 +14827,31 @@
       </c>
       <c r="C46" s="47">
         <f>SUM(C40:C45)/6</f>
-        <v>0.36751784016636962</v>
+        <v>0.57193450683303626</v>
       </c>
       <c r="D46" s="47">
         <f>SUM(D40:D45)/6</f>
-        <v>0.5033333333333333</v>
+        <v>0.89</v>
       </c>
       <c r="E46" s="47">
         <f>SUM(E40:E45)/6</f>
-        <v>0.49666666666666676</v>
+        <v>0.11</v>
       </c>
       <c r="F46" s="47">
-        <f>IFERROR(IF((0.7-$C46)/$E46&gt;0,(0.7-$C46)/$E46,0), IF($C46&gt;=0.7, 0, 1))</f>
-        <v>0.66942716745026232</v>
+        <f t="shared" si="49"/>
+        <v>1.1642317560633064</v>
       </c>
       <c r="G46" s="47">
-        <f t="shared" si="49"/>
-        <v>0.46808488557106775</v>
+        <f t="shared" si="50"/>
+        <v>0.25514084697239742</v>
       </c>
       <c r="H46" s="47">
-        <f t="shared" si="50"/>
-        <v>0.26674260369187319</v>
+        <f t="shared" si="51"/>
+        <v>0</v>
       </c>
       <c r="I46" s="47">
-        <f>IFERROR(IF((0.4-$C46)/$E46&gt;0,(0.4-$C46)/$E46,0), IF($C46&gt;=0.4, 0, 1))</f>
-        <v>6.5400321812678644E-2</v>
+        <f t="shared" si="52"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>